<commit_message>
fix: đồng bộ email Google trong nhập user
</commit_message>
<xml_diff>
--- a/public/templates/mau-nhap-nguoi-dung.xlsx
+++ b/public/templates/mau-nhap-nguoi-dung.xlsx
@@ -530,6 +530,7 @@
     <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -571,6 +572,9 @@
       </x:c>
       <x:c r="M1" s="11" t="str">
         <x:v>Ghi chú</x:v>
+      </x:c>
+      <x:c r="N1" s="11" t="str">
+        <x:v>Email Google Workspace</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="23" customHeight="1">
@@ -587,6 +591,7 @@
       <x:c r="K2" s="28"/>
       <x:c r="L2" s="30"/>
       <x:c r="M2" s="37"/>
+      <x:c r="N2" s="38"/>
     </x:row>
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="31"/>
@@ -602,6 +607,7 @@
       <x:c r="K3" s="31"/>
       <x:c r="L3" s="33"/>
       <x:c r="M3" s="38"/>
+      <x:c r="N3" s="38"/>
     </x:row>
     <x:row r="4" ht="23" customHeight="1">
       <x:c r="A4" s="31"/>
@@ -617,6 +623,7 @@
       <x:c r="K4" s="31"/>
       <x:c r="L4" s="33"/>
       <x:c r="M4" s="38"/>
+      <x:c r="N4" s="38"/>
     </x:row>
     <x:row r="5" ht="23" customHeight="1">
       <x:c r="A5" s="31"/>
@@ -632,6 +639,7 @@
       <x:c r="K5" s="31"/>
       <x:c r="L5" s="33"/>
       <x:c r="M5" s="38"/>
+      <x:c r="N5" s="38"/>
     </x:row>
     <x:row r="6" ht="23" customHeight="1">
       <x:c r="A6" s="31"/>
@@ -647,6 +655,7 @@
       <x:c r="K6" s="31"/>
       <x:c r="L6" s="33"/>
       <x:c r="M6" s="38"/>
+      <x:c r="N6" s="38"/>
     </x:row>
     <x:row r="7" ht="23" customHeight="1">
       <x:c r="A7" s="31"/>
@@ -662,6 +671,7 @@
       <x:c r="K7" s="31"/>
       <x:c r="L7" s="33"/>
       <x:c r="M7" s="38"/>
+      <x:c r="N7" s="38"/>
     </x:row>
     <x:row r="8" ht="23" customHeight="1">
       <x:c r="A8" s="31"/>
@@ -677,6 +687,7 @@
       <x:c r="K8" s="31"/>
       <x:c r="L8" s="33"/>
       <x:c r="M8" s="38"/>
+      <x:c r="N8" s="38"/>
     </x:row>
     <x:row r="9" ht="23" customHeight="1">
       <x:c r="A9" s="31"/>
@@ -692,6 +703,7 @@
       <x:c r="K9" s="31"/>
       <x:c r="L9" s="33"/>
       <x:c r="M9" s="38"/>
+      <x:c r="N9" s="38"/>
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
       <x:c r="A10" s="31"/>
@@ -707,6 +719,7 @@
       <x:c r="K10" s="31"/>
       <x:c r="L10" s="33"/>
       <x:c r="M10" s="38"/>
+      <x:c r="N10" s="38"/>
     </x:row>
     <x:row r="11" ht="23" customHeight="1">
       <x:c r="A11" s="31"/>
@@ -722,6 +735,7 @@
       <x:c r="K11" s="31"/>
       <x:c r="L11" s="33"/>
       <x:c r="M11" s="38"/>
+      <x:c r="N11" s="38"/>
     </x:row>
     <x:row r="12" ht="23" customHeight="1">
       <x:c r="A12" s="31"/>
@@ -737,6 +751,7 @@
       <x:c r="K12" s="31"/>
       <x:c r="L12" s="33"/>
       <x:c r="M12" s="38"/>
+      <x:c r="N12" s="38"/>
     </x:row>
     <x:row r="13" ht="23" customHeight="1">
       <x:c r="A13" s="31"/>
@@ -752,6 +767,7 @@
       <x:c r="K13" s="31"/>
       <x:c r="L13" s="33"/>
       <x:c r="M13" s="38"/>
+      <x:c r="N13" s="38"/>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
       <x:c r="A14" s="31"/>
@@ -767,6 +783,7 @@
       <x:c r="K14" s="31"/>
       <x:c r="L14" s="33"/>
       <x:c r="M14" s="38"/>
+      <x:c r="N14" s="38"/>
     </x:row>
     <x:row r="15" ht="23" customHeight="1">
       <x:c r="A15" s="31"/>
@@ -782,6 +799,7 @@
       <x:c r="K15" s="31"/>
       <x:c r="L15" s="33"/>
       <x:c r="M15" s="38"/>
+      <x:c r="N15" s="38"/>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
       <x:c r="A16" s="31"/>
@@ -797,6 +815,7 @@
       <x:c r="K16" s="31"/>
       <x:c r="L16" s="33"/>
       <x:c r="M16" s="38"/>
+      <x:c r="N16" s="38"/>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
       <x:c r="A17" s="31"/>
@@ -812,6 +831,7 @@
       <x:c r="K17" s="31"/>
       <x:c r="L17" s="33"/>
       <x:c r="M17" s="38"/>
+      <x:c r="N17" s="38"/>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
       <x:c r="A18" s="31"/>
@@ -827,6 +847,7 @@
       <x:c r="K18" s="31"/>
       <x:c r="L18" s="33"/>
       <x:c r="M18" s="38"/>
+      <x:c r="N18" s="38"/>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
       <x:c r="A19" s="31"/>
@@ -842,6 +863,7 @@
       <x:c r="K19" s="31"/>
       <x:c r="L19" s="33"/>
       <x:c r="M19" s="38"/>
+      <x:c r="N19" s="38"/>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
       <x:c r="A20" s="31"/>
@@ -857,6 +879,7 @@
       <x:c r="K20" s="31"/>
       <x:c r="L20" s="33"/>
       <x:c r="M20" s="38"/>
+      <x:c r="N20" s="38"/>
     </x:row>
     <x:row r="21" ht="23" customHeight="1">
       <x:c r="A21" s="31"/>
@@ -872,6 +895,7 @@
       <x:c r="K21" s="31"/>
       <x:c r="L21" s="33"/>
       <x:c r="M21" s="38"/>
+      <x:c r="N21" s="38"/>
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
       <x:c r="A22" s="31"/>
@@ -887,6 +911,7 @@
       <x:c r="K22" s="31"/>
       <x:c r="L22" s="33"/>
       <x:c r="M22" s="38"/>
+      <x:c r="N22" s="38"/>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
       <x:c r="A23" s="31"/>
@@ -902,6 +927,7 @@
       <x:c r="K23" s="31"/>
       <x:c r="L23" s="33"/>
       <x:c r="M23" s="38"/>
+      <x:c r="N23" s="38"/>
     </x:row>
     <x:row r="24" ht="23" customHeight="1">
       <x:c r="A24" s="31"/>
@@ -917,6 +943,7 @@
       <x:c r="K24" s="31"/>
       <x:c r="L24" s="33"/>
       <x:c r="M24" s="38"/>
+      <x:c r="N24" s="38"/>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
       <x:c r="A25" s="31"/>
@@ -932,6 +959,7 @@
       <x:c r="K25" s="31"/>
       <x:c r="L25" s="33"/>
       <x:c r="M25" s="38"/>
+      <x:c r="N25" s="38"/>
     </x:row>
     <x:row r="26" ht="23" customHeight="1">
       <x:c r="A26" s="31"/>
@@ -947,6 +975,7 @@
       <x:c r="K26" s="31"/>
       <x:c r="L26" s="33"/>
       <x:c r="M26" s="38"/>
+      <x:c r="N26" s="38"/>
     </x:row>
     <x:row r="27" ht="23" customHeight="1">
       <x:c r="A27" s="31"/>
@@ -962,6 +991,7 @@
       <x:c r="K27" s="31"/>
       <x:c r="L27" s="33"/>
       <x:c r="M27" s="38"/>
+      <x:c r="N27" s="38"/>
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
       <x:c r="A28" s="31"/>
@@ -977,6 +1007,7 @@
       <x:c r="K28" s="31"/>
       <x:c r="L28" s="33"/>
       <x:c r="M28" s="38"/>
+      <x:c r="N28" s="38"/>
     </x:row>
     <x:row r="29" ht="23" customHeight="1">
       <x:c r="A29" s="31"/>
@@ -992,6 +1023,7 @@
       <x:c r="K29" s="31"/>
       <x:c r="L29" s="33"/>
       <x:c r="M29" s="38"/>
+      <x:c r="N29" s="38"/>
     </x:row>
     <x:row r="30" ht="23" customHeight="1">
       <x:c r="A30" s="31"/>
@@ -1007,6 +1039,7 @@
       <x:c r="K30" s="31"/>
       <x:c r="L30" s="33"/>
       <x:c r="M30" s="38"/>
+      <x:c r="N30" s="38"/>
     </x:row>
     <x:row r="31" ht="23" customHeight="1">
       <x:c r="A31" s="31"/>
@@ -1022,6 +1055,7 @@
       <x:c r="K31" s="31"/>
       <x:c r="L31" s="33"/>
       <x:c r="M31" s="38"/>
+      <x:c r="N31" s="38"/>
     </x:row>
     <x:row r="32" ht="23" customHeight="1">
       <x:c r="A32" s="31"/>
@@ -1037,6 +1071,7 @@
       <x:c r="K32" s="31"/>
       <x:c r="L32" s="33"/>
       <x:c r="M32" s="38"/>
+      <x:c r="N32" s="38"/>
     </x:row>
     <x:row r="33" ht="23" customHeight="1">
       <x:c r="A33" s="31"/>
@@ -1052,6 +1087,7 @@
       <x:c r="K33" s="31"/>
       <x:c r="L33" s="33"/>
       <x:c r="M33" s="38"/>
+      <x:c r="N33" s="38"/>
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
       <x:c r="A34" s="31"/>
@@ -1067,6 +1103,7 @@
       <x:c r="K34" s="31"/>
       <x:c r="L34" s="33"/>
       <x:c r="M34" s="38"/>
+      <x:c r="N34" s="38"/>
     </x:row>
     <x:row r="35" ht="23" customHeight="1">
       <x:c r="A35" s="31"/>
@@ -1082,6 +1119,7 @@
       <x:c r="K35" s="31"/>
       <x:c r="L35" s="33"/>
       <x:c r="M35" s="38"/>
+      <x:c r="N35" s="38"/>
     </x:row>
     <x:row r="36" ht="23" customHeight="1">
       <x:c r="A36" s="31"/>
@@ -1097,6 +1135,7 @@
       <x:c r="K36" s="31"/>
       <x:c r="L36" s="33"/>
       <x:c r="M36" s="38"/>
+      <x:c r="N36" s="38"/>
     </x:row>
     <x:row r="37" ht="23" customHeight="1">
       <x:c r="A37" s="31"/>
@@ -1112,6 +1151,7 @@
       <x:c r="K37" s="31"/>
       <x:c r="L37" s="33"/>
       <x:c r="M37" s="38"/>
+      <x:c r="N37" s="38"/>
     </x:row>
     <x:row r="38" ht="23" customHeight="1">
       <x:c r="A38" s="31"/>
@@ -1127,6 +1167,7 @@
       <x:c r="K38" s="31"/>
       <x:c r="L38" s="33"/>
       <x:c r="M38" s="38"/>
+      <x:c r="N38" s="38"/>
     </x:row>
     <x:row r="39" ht="23" customHeight="1">
       <x:c r="A39" s="31"/>
@@ -1142,6 +1183,7 @@
       <x:c r="K39" s="31"/>
       <x:c r="L39" s="33"/>
       <x:c r="M39" s="38"/>
+      <x:c r="N39" s="38"/>
     </x:row>
     <x:row r="40" ht="23" customHeight="1">
       <x:c r="A40" s="31"/>
@@ -1157,6 +1199,7 @@
       <x:c r="K40" s="31"/>
       <x:c r="L40" s="33"/>
       <x:c r="M40" s="38"/>
+      <x:c r="N40" s="38"/>
     </x:row>
     <x:row r="41" ht="23" customHeight="1">
       <x:c r="A41" s="31"/>
@@ -1172,6 +1215,7 @@
       <x:c r="K41" s="31"/>
       <x:c r="L41" s="33"/>
       <x:c r="M41" s="38"/>
+      <x:c r="N41" s="38"/>
     </x:row>
     <x:row r="42" ht="23" customHeight="1">
       <x:c r="A42" s="31"/>
@@ -1187,6 +1231,7 @@
       <x:c r="K42" s="31"/>
       <x:c r="L42" s="33"/>
       <x:c r="M42" s="38"/>
+      <x:c r="N42" s="38"/>
     </x:row>
     <x:row r="43" ht="23" customHeight="1">
       <x:c r="A43" s="31"/>
@@ -1202,6 +1247,7 @@
       <x:c r="K43" s="31"/>
       <x:c r="L43" s="33"/>
       <x:c r="M43" s="38"/>
+      <x:c r="N43" s="38"/>
     </x:row>
     <x:row r="44" ht="23" customHeight="1">
       <x:c r="A44" s="31"/>
@@ -1217,6 +1263,7 @@
       <x:c r="K44" s="31"/>
       <x:c r="L44" s="33"/>
       <x:c r="M44" s="38"/>
+      <x:c r="N44" s="38"/>
     </x:row>
     <x:row r="45" ht="23" customHeight="1">
       <x:c r="A45" s="31"/>
@@ -1232,6 +1279,7 @@
       <x:c r="K45" s="31"/>
       <x:c r="L45" s="33"/>
       <x:c r="M45" s="38"/>
+      <x:c r="N45" s="38"/>
     </x:row>
     <x:row r="46" ht="23" customHeight="1">
       <x:c r="A46" s="31"/>
@@ -1247,6 +1295,7 @@
       <x:c r="K46" s="31"/>
       <x:c r="L46" s="33"/>
       <x:c r="M46" s="38"/>
+      <x:c r="N46" s="38"/>
     </x:row>
     <x:row r="47" ht="23" customHeight="1">
       <x:c r="A47" s="31"/>
@@ -1262,6 +1311,7 @@
       <x:c r="K47" s="31"/>
       <x:c r="L47" s="33"/>
       <x:c r="M47" s="38"/>
+      <x:c r="N47" s="38"/>
     </x:row>
     <x:row r="48" ht="23" customHeight="1">
       <x:c r="A48" s="31"/>
@@ -1277,6 +1327,7 @@
       <x:c r="K48" s="31"/>
       <x:c r="L48" s="33"/>
       <x:c r="M48" s="38"/>
+      <x:c r="N48" s="38"/>
     </x:row>
     <x:row r="49" ht="23" customHeight="1">
       <x:c r="A49" s="31"/>
@@ -1292,6 +1343,7 @@
       <x:c r="K49" s="31"/>
       <x:c r="L49" s="33"/>
       <x:c r="M49" s="38"/>
+      <x:c r="N49" s="38"/>
     </x:row>
     <x:row r="50" ht="23" customHeight="1">
       <x:c r="A50" s="31"/>
@@ -1307,6 +1359,7 @@
       <x:c r="K50" s="31"/>
       <x:c r="L50" s="33"/>
       <x:c r="M50" s="38"/>
+      <x:c r="N50" s="38"/>
     </x:row>
     <x:row r="51" ht="23" customHeight="1">
       <x:c r="A51" s="34"/>
@@ -1322,6 +1375,7 @@
       <x:c r="K51" s="34"/>
       <x:c r="L51" s="36"/>
       <x:c r="M51" s="39"/>
+      <x:c r="N51" s="39"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
@@ -1557,7 +1611,7 @@
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
       <x:c r="A8" s="60" t="str">
-        <x:v>6. Việc cho phép đăng nhập Google không tự động: cấu hình OAuth/test user/domain vẫn thực hiện thủ công trên Google Cloud.</x:v>
+        <x:v>6. Email Google Workspace chỉ dùng để cấp quyền xem file đính kèm; OAuth Google Drive vẫn do quản trị viên kết nối thủ công.</x:v>
       </x:c>
       <x:c r="B8" s="60"/>
       <x:c r="C8" s="60"/>

</xml_diff>